<commit_message>
docs: update Wonderpin brand colors
</commit_message>
<xml_diff>
--- a/outputs/weekly-wonderpin-20260716/weekly-wonderpin-program-candidates.xlsx
+++ b/outputs/weekly-wonderpin-20260716/weekly-wonderpin-program-candidates.xlsx
@@ -2,10 +2,10 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="사용 안내" sheetId="1" r:id="Ra53ca573c7e24d02"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="프로그램 후보" sheetId="2" r:id="R8c0dfebb9d5f4090"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="발행 전 재확인" sheetId="3" r:id="R27a92ad99a2c4d8f"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="데이터 사전" sheetId="4" r:id="R61bd448ec89c42a4"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="사용 안내" sheetId="1" r:id="R4ae10ea4dd3a457a"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="프로그램 후보" sheetId="2" r:id="R95fdde7cb1f24ec5"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="발행 전 재확인" sheetId="3" r:id="Rae6589e67a1141c6"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="데이터 사전" sheetId="4" r:id="R1a6ddf792bc34c54"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -32,19 +32,19 @@
     </x:font>
     <x:font>
       <x:sz val="11"/>
-      <x:color rgb="FF27242D"/>
+      <x:color rgb="FF1D2A3A"/>
       <x:name val="Carlito"/>
     </x:font>
     <x:font>
       <x:b/>
       <x:sz val="11"/>
-      <x:color rgb="FF5A3FA3"/>
+      <x:color rgb="FF0167D3"/>
       <x:name val="Carlito"/>
     </x:font>
     <x:font>
       <x:b/>
       <x:sz val="14"/>
-      <x:color rgb="FF27242D"/>
+      <x:color rgb="FF1D2A3A"/>
       <x:name val="Carlito"/>
     </x:font>
     <x:font>
@@ -56,7 +56,7 @@
     <x:font>
       <x:b/>
       <x:sz val="11"/>
-      <x:color rgb="FF27242D"/>
+      <x:color rgb="FF1D2A3A"/>
       <x:name val="Carlito"/>
     </x:font>
   </x:fonts>
@@ -69,17 +69,17 @@
     </x:fill>
     <x:fill>
       <x:patternFill patternType="solid">
-        <x:fgColor rgb="FF5A3FA3"/>
+        <x:fgColor rgb="FF0167D3"/>
       </x:patternFill>
     </x:fill>
     <x:fill>
       <x:patternFill patternType="solid">
-        <x:fgColor rgb="FFFDECF0"/>
+        <x:fgColor rgb="FFFFF8DD"/>
       </x:patternFill>
     </x:fill>
     <x:fill>
       <x:patternFill patternType="solid">
-        <x:fgColor rgb="FFF2EFFA"/>
+        <x:fgColor rgb="FFEAF4FF"/>
       </x:patternFill>
     </x:fill>
     <x:fill>
@@ -92,110 +92,110 @@
     <x:border/>
     <x:border>
       <x:left style="thin">
-        <x:color rgb="FFF28CA6"/>
+        <x:color rgb="FFF3B806"/>
       </x:left>
       <x:top style="thin">
-        <x:color rgb="FFF28CA6"/>
+        <x:color rgb="FFF3B806"/>
       </x:top>
     </x:border>
     <x:border>
       <x:top style="thin">
-        <x:color rgb="FFF28CA6"/>
+        <x:color rgb="FFF3B806"/>
       </x:top>
     </x:border>
     <x:border>
       <x:right style="thin">
-        <x:color rgb="FFF28CA6"/>
+        <x:color rgb="FFF3B806"/>
       </x:right>
       <x:top style="thin">
-        <x:color rgb="FFF28CA6"/>
+        <x:color rgb="FFF3B806"/>
       </x:top>
     </x:border>
     <x:border>
       <x:left style="thin">
-        <x:color rgb="FFF28CA6"/>
+        <x:color rgb="FFF3B806"/>
       </x:left>
       <x:bottom style="thin">
-        <x:color rgb="FFF28CA6"/>
+        <x:color rgb="FFF3B806"/>
       </x:bottom>
     </x:border>
     <x:border>
       <x:bottom style="thin">
-        <x:color rgb="FFF28CA6"/>
+        <x:color rgb="FFF3B806"/>
       </x:bottom>
     </x:border>
     <x:border>
       <x:right style="thin">
-        <x:color rgb="FFF28CA6"/>
+        <x:color rgb="FFF3B806"/>
       </x:right>
       <x:bottom style="thin">
-        <x:color rgb="FFF28CA6"/>
+        <x:color rgb="FFF3B806"/>
       </x:bottom>
     </x:border>
     <x:border>
       <x:left style="thin">
-        <x:color rgb="FFDDD8E8"/>
+        <x:color rgb="FFD7E3F2"/>
       </x:left>
       <x:top style="thin">
-        <x:color rgb="FFDDD8E8"/>
+        <x:color rgb="FFD7E3F2"/>
       </x:top>
       <x:bottom style="thin">
-        <x:color rgb="FFDDD8E8"/>
+        <x:color rgb="FFD7E3F2"/>
       </x:bottom>
     </x:border>
     <x:border>
       <x:right style="thin">
-        <x:color rgb="FFDDD8E8"/>
+        <x:color rgb="FFD7E3F2"/>
       </x:right>
       <x:top style="thin">
-        <x:color rgb="FFDDD8E8"/>
+        <x:color rgb="FFD7E3F2"/>
       </x:top>
       <x:bottom style="thin">
-        <x:color rgb="FFDDD8E8"/>
+        <x:color rgb="FFD7E3F2"/>
       </x:bottom>
     </x:border>
     <x:border>
       <x:left style="thin">
-        <x:color rgb="FFF28CA6"/>
+        <x:color rgb="FFF3B806"/>
       </x:left>
       <x:top style="thin">
-        <x:color rgb="FFF28CA6"/>
+        <x:color rgb="FFF3B806"/>
       </x:top>
       <x:bottom style="thin">
-        <x:color rgb="FFF28CA6"/>
+        <x:color rgb="FFF3B806"/>
       </x:bottom>
     </x:border>
     <x:border>
       <x:top style="thin">
-        <x:color rgb="FFF28CA6"/>
+        <x:color rgb="FFF3B806"/>
       </x:top>
       <x:bottom style="thin">
-        <x:color rgb="FFF28CA6"/>
+        <x:color rgb="FFF3B806"/>
       </x:bottom>
     </x:border>
     <x:border>
       <x:right style="thin">
-        <x:color rgb="FFF28CA6"/>
+        <x:color rgb="FFF3B806"/>
       </x:right>
       <x:top style="thin">
-        <x:color rgb="FFF28CA6"/>
+        <x:color rgb="FFF3B806"/>
       </x:top>
       <x:bottom style="thin">
-        <x:color rgb="FFF28CA6"/>
+        <x:color rgb="FFF3B806"/>
       </x:bottom>
     </x:border>
     <x:border>
       <x:left style="thin">
-        <x:color rgb="FFDDD8E8"/>
+        <x:color rgb="FFD7E3F2"/>
       </x:left>
       <x:right style="thin">
-        <x:color rgb="FFDDD8E8"/>
+        <x:color rgb="FFD7E3F2"/>
       </x:right>
       <x:top style="thin">
-        <x:color rgb="FFDDD8E8"/>
+        <x:color rgb="FFD7E3F2"/>
       </x:top>
       <x:bottom style="thin">
-        <x:color rgb="FFDDD8E8"/>
+        <x:color rgb="FFD7E3F2"/>
       </x:bottom>
     </x:border>
     <x:border>
@@ -361,21 +361,21 @@
   <x:dxfs count="4">
     <x:dxf>
       <x:font>
-        <x:color rgb="FF5A3FA3"/>
+        <x:color rgb="FF0167D3"/>
       </x:font>
       <x:fill>
         <x:patternFill patternType="solid">
-          <x:bgColor rgb="FFF2EFFA"/>
+          <x:bgColor rgb="FFEAF4FF"/>
         </x:patternFill>
       </x:fill>
     </x:dxf>
     <x:dxf>
       <x:font>
-        <x:color rgb="FF27242D"/>
+        <x:color rgb="FF1D2A3A"/>
       </x:font>
       <x:fill>
         <x:patternFill patternType="solid">
-          <x:bgColor rgb="FFFDECF0"/>
+          <x:bgColor rgb="FFFFF8DD"/>
         </x:patternFill>
       </x:fill>
     </x:dxf>
@@ -393,11 +393,11 @@
     <x:dxf>
       <x:font>
         <x:b/>
-        <x:color rgb="FF27242D"/>
+        <x:color rgb="FF1D2A3A"/>
       </x:font>
       <x:fill>
         <x:patternFill patternType="solid">
-          <x:bgColor rgb="FFFDECF0"/>
+          <x:bgColor rgb="FFFFF8DD"/>
         </x:patternFill>
       </x:fill>
     </x:dxf>
@@ -9062,7 +9062,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R729f0e86a86a457e"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rf776d528e4e74281"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -11965,7 +11965,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R378055a443cc4a73"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R45e54e7b4d244dae"/>
   </x:tableParts>
 </x:worksheet>
 </file>

</xml_diff>